<commit_message>
Implemedted the Banking app topic taught on 6 Sep
</commit_message>
<xml_diff>
--- a/bank_records_1.xlsx
+++ b/bank_records_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,47 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Date-Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345456677</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> chin</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1122</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1f3d2977</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:56:34</t>
         </is>
       </c>
     </row>

</xml_diff>